<commit_message>
Add Netlify + backend deployment wiring for live XGBoost dashboard
</commit_message>
<xml_diff>
--- a/outputs/multi_city/tables/multi_city_analysis_summary.xlsx
+++ b/outputs/multi_city/tables/multi_city_analysis_summary.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pooled_quantile" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cross_city_tests" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="xgboost_city_metrics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="xgboost_tuning_summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,13 +461,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.443145001393529</v>
+        <v>4.4431450013941</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="3">
@@ -476,13 +477,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.08319622817396245</v>
+        <v>0.08319622817371827</v>
       </c>
       <c r="C3" t="n">
-        <v>4.157225473495323e-07</v>
+        <v>4.15722547380059e-07</v>
       </c>
       <c r="D3" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="4">
@@ -492,13 +493,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5648283513422838</v>
+        <v>0.5648283513414091</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="5">
@@ -508,13 +509,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1290061679269675</v>
+        <v>0.129006167927103</v>
       </c>
       <c r="C5" t="n">
-        <v>1.768335830571189e-13</v>
+        <v>1.768335830545145e-13</v>
       </c>
       <c r="D5" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="6">
@@ -524,13 +525,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.00175826147361974</v>
+        <v>0.001758261473381694</v>
       </c>
       <c r="C6" t="n">
-        <v>0.921528295662125</v>
+        <v>0.9215282956727615</v>
       </c>
       <c r="D6" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="7">
@@ -540,13 +541,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3416981393909595</v>
+        <v>0.3416981393907812</v>
       </c>
       <c r="C7" t="n">
-        <v>9.658517254699228e-175</v>
+        <v>9.658517252542154e-175</v>
       </c>
       <c r="D7" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="8">
@@ -556,13 +557,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.5650125737465571</v>
+        <v>0.5650125737472401</v>
       </c>
       <c r="C8" t="n">
-        <v>4.845193483051645e-109</v>
+        <v>4.845193483037293e-109</v>
       </c>
       <c r="D8" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="9">
@@ -572,13 +573,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.6337375435950526</v>
+        <v>-0.6337375435952312</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="10">
@@ -588,13 +589,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.230247678578668</v>
+        <v>-1.230247678578918</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="11">
@@ -604,13 +605,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1165488572791486</v>
+        <v>0.1165488572791514</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="12">
@@ -620,13 +621,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.01698325177184844</v>
+        <v>-0.01698325177185978</v>
       </c>
       <c r="C12" t="n">
-        <v>1.12942710327945e-19</v>
+        <v>1.129427103253205e-19</v>
       </c>
       <c r="D12" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="13">
@@ -636,13 +637,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.1075412741755082</v>
+        <v>-0.1075412741755148</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="14">
@@ -652,13 +653,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.05470865909874665</v>
+        <v>-0.05470865909877329</v>
       </c>
       <c r="C14" t="n">
-        <v>6.371491062902286e-248</v>
+        <v>6.371491062526016e-248</v>
       </c>
       <c r="D14" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="15">
@@ -668,13 +669,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.0001050659269690984</v>
+        <v>-0.000105065926965753</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9557334698758153</v>
+        <v>0.9557334698772162</v>
       </c>
       <c r="D15" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="16">
@@ -684,13 +685,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.02266158123625369</v>
+        <v>-0.0226615812362542</v>
       </c>
       <c r="C16" t="n">
-        <v>4.159980864129359e-41</v>
+        <v>4.159980864110577e-41</v>
       </c>
       <c r="D16" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="17">
@@ -700,13 +701,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0001103763536456757</v>
+        <v>0.0001103763536451714</v>
       </c>
       <c r="C17" t="n">
-        <v>9.245257058381444e-35</v>
+        <v>9.245257064760728e-35</v>
       </c>
       <c r="D17" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="18">
@@ -716,13 +717,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.0001491096054681639</v>
+        <v>-0.0001491096054682352</v>
       </c>
       <c r="C18" t="n">
-        <v>9.914300614825378e-30</v>
+        <v>9.914300614222562e-30</v>
       </c>
       <c r="D18" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="19">
@@ -732,13 +733,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-0.000880991624289492</v>
+        <v>-0.0008809916242881155</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0001804860115982252</v>
+        <v>0.0001804860116022679</v>
       </c>
       <c r="D19" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="20">
@@ -748,13 +749,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.00412821803571433</v>
+        <v>0.004128218035713475</v>
       </c>
       <c r="C20" t="n">
-        <v>3.990504244582361e-28</v>
+        <v>3.990504244658425e-28</v>
       </c>
       <c r="D20" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="21">
@@ -764,13 +765,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.001441859262833202</v>
+        <v>0.001441859262831513</v>
       </c>
       <c r="C21" t="n">
-        <v>2.289624265048175e-08</v>
+        <v>2.289624265130298e-08</v>
       </c>
       <c r="D21" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="22">
@@ -780,13 +781,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.003421966833922912</v>
+        <v>0.003421966833921263</v>
       </c>
       <c r="C22" t="n">
-        <v>1.066286278414698e-20</v>
+        <v>1.066286278457212e-20</v>
       </c>
       <c r="D22" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="23">
@@ -796,13 +797,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.0006545664605282465</v>
+        <v>0.0006545664605265909</v>
       </c>
       <c r="C23" t="n">
-        <v>0.09184630478900636</v>
+        <v>0.09184630478981877</v>
       </c>
       <c r="D23" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="24">
@@ -812,13 +813,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.006478097955521464</v>
+        <v>0.006478097955520199</v>
       </c>
       <c r="C24" t="n">
-        <v>3.161960577824749e-123</v>
+        <v>3.161960578087814e-123</v>
       </c>
       <c r="D24" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
     <row r="25">
@@ -828,13 +829,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.0004092279085986001</v>
+        <v>0.0004092279085984558</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>0.572493083374196</v>
+        <v>0.5724930833741959</v>
       </c>
     </row>
   </sheetData>
@@ -883,7 +884,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.098536185243006</v>
+        <v>4.098536168520923</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -899,7 +900,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1256561640949485</v>
+        <v>0.1256563783468891</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -915,7 +916,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.008107701988024</v>
+        <v>1.008107732516123</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -931,7 +932,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.2907717148414122</v>
+        <v>0.2907716982534794</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -947,7 +948,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.1027353599108665</v>
+        <v>-0.1027353571647609</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -963,7 +964,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9643290009839802</v>
+        <v>0.9643289834741609</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -979,7 +980,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.3287980502713594</v>
+        <v>0.3287980634171106</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -995,7 +996,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.7432151549768093</v>
+        <v>-0.7432151548240213</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -1011,7 +1012,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-1.45660208818029</v>
+        <v>-1.456602102031923</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -1027,7 +1028,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.09617352086884789</v>
+        <v>0.09617351918172679</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -1043,7 +1044,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.01523127935914914</v>
+        <v>-0.01523129547254598</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -1059,7 +1060,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.09347327142165351</v>
+        <v>-0.09347326382680876</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -1075,7 +1076,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.04664975477204703</v>
+        <v>-0.04664975299367491</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -1091,7 +1092,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.01201715031154293</v>
+        <v>0.01201715253792646</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -1107,7 +1108,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.08001499606762774</v>
+        <v>-0.08001498507698335</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -1123,10 +1124,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-1.298397652998995e-05</v>
+        <v>-1.298390070572641e-05</v>
       </c>
       <c r="D17" t="n">
-        <v>7.44028555195493e-116</v>
+        <v>7.461393506722341e-116</v>
       </c>
     </row>
     <row r="18">
@@ -1139,10 +1140,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-3.242665381736343e-06</v>
+        <v>-3.242625837784896e-06</v>
       </c>
       <c r="D18" t="n">
-        <v>6.253794063075039e-05</v>
+        <v>6.255039897511553e-05</v>
       </c>
     </row>
     <row r="19">
@@ -1155,7 +1156,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.001498306530562488</v>
+        <v>0.001498306710949748</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -1171,7 +1172,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.003909229905886491</v>
+        <v>0.003909228479242799</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -1187,7 +1188,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-0.00146315826190424</v>
+        <v>-0.001463159731015296</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -1203,7 +1204,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.001735742177528365</v>
+        <v>0.001735742177590538</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
@@ -1219,7 +1220,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.001589155950169285</v>
+        <v>0.001589155311721768</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -1235,7 +1236,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-0.002235277773843691</v>
+        <v>-0.002235278449962408</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -1251,7 +1252,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.0002993101920153798</v>
+        <v>0.0002993101911952945</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -1267,7 +1268,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4.322580099862535</v>
+        <v>4.322580066858791</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -1283,7 +1284,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.2739777849055827</v>
+        <v>0.2739778301329352</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -1299,7 +1300,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.7546389081981033</v>
+        <v>0.7546389411436394</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -1315,7 +1316,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.5347723293816671</v>
+        <v>0.5347723593586124</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -1331,7 +1332,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.1702506349538453</v>
+        <v>0.1702506688889116</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -1347,7 +1348,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.7028447074699216</v>
+        <v>0.7028449205681682</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -1363,7 +1364,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.3250163422208061</v>
+        <v>0.3250163411685207</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -1379,7 +1380,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-0.729651376220616</v>
+        <v>-0.7296513763196657</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1395,7 +1396,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-1.441071017679157</v>
+        <v>-1.441071017748477</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1411,7 +1412,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.1194714242785722</v>
+        <v>0.1194714244334136</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1427,7 +1428,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>-0.0386354855894524</v>
+        <v>-0.03863548591544941</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
@@ -1443,7 +1444,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>-0.1129628193490362</v>
+        <v>-0.1129628195243413</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1459,7 +1460,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-0.08577292090984656</v>
+        <v>-0.08577292105366041</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -1475,7 +1476,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>-0.01484154923042524</v>
+        <v>-0.01484154954027872</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1491,7 +1492,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-0.08991722069890784</v>
+        <v>-0.08991745662632411</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1507,10 +1508,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1.197862829760421e-09</v>
+        <v>1.197972006317105e-09</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9968722607119895</v>
+        <v>0.9968719706223539</v>
       </c>
     </row>
     <row r="42">
@@ -1523,10 +1524,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>-1.632064188655802e-09</v>
+        <v>-1.632202924900517e-09</v>
       </c>
       <c r="D42" t="n">
-        <v>0.9970954037231607</v>
+        <v>0.9970951521523332</v>
       </c>
     </row>
     <row r="43">
@@ -1539,7 +1540,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.0003828476674243575</v>
+        <v>0.0003828483331744792</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
@@ -1555,7 +1556,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.002890296713303542</v>
+        <v>0.002890295843826607</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
@@ -1571,7 +1572,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>-0.00038282902642095</v>
+        <v>-0.0003828296958090505</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -1587,7 +1588,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.000528618807948078</v>
+        <v>0.0005286181876726914</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
@@ -1603,10 +1604,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>-0.0003828389490081463</v>
+        <v>-0.0003828396256722044</v>
       </c>
       <c r="D47" t="n">
-        <v>1.303104922429084e-183</v>
+        <v>1.299449107418606e-183</v>
       </c>
     </row>
     <row r="48">
@@ -1619,10 +1620,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2.460621908539906e-05</v>
+        <v>2.462646989442874e-05</v>
       </c>
       <c r="D48" t="n">
-        <v>0.00838852993955579</v>
+        <v>0.008334949213520281</v>
       </c>
     </row>
     <row r="49">
@@ -1635,7 +1636,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.0005360268363296672</v>
+        <v>0.0005360268363976128</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -1651,7 +1652,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4.450209710731542</v>
+        <v>4.450210973002811</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -1667,10 +1668,10 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.04564307555313007</v>
+        <v>0.04564257378501679</v>
       </c>
       <c r="D51" t="n">
-        <v>6.061348418892513e-42</v>
+        <v>6.076867482915123e-42</v>
       </c>
     </row>
     <row r="52">
@@ -1683,7 +1684,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.2409271513056694</v>
+        <v>0.2409266965108543</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
@@ -1699,10 +1700,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.09338034962684105</v>
+        <v>0.09337842806030494</v>
       </c>
       <c r="D53" t="n">
-        <v>5.962035216273716e-143</v>
+        <v>6.05304789495267e-143</v>
       </c>
     </row>
     <row r="54">
@@ -1715,10 +1716,10 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.01986690080462949</v>
+        <v>0.0198663971282258</v>
       </c>
       <c r="D54" t="n">
-        <v>1.232581497126346e-07</v>
+        <v>1.233585939922516e-07</v>
       </c>
     </row>
     <row r="55">
@@ -1731,10 +1732,10 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>-0.04913874153061215</v>
+        <v>-0.04914266220015406</v>
       </c>
       <c r="D55" t="n">
-        <v>8.831649514017318e-89</v>
+        <v>8.564329905782184e-89</v>
       </c>
     </row>
     <row r="56">
@@ -1747,10 +1748,10 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.0730935762076399</v>
+        <v>0.07334089528704624</v>
       </c>
       <c r="D56" t="n">
-        <v>4.130183393819508e-38</v>
+        <v>2.342623424630981e-38</v>
       </c>
     </row>
     <row r="57">
@@ -1763,7 +1764,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>-0.6102243613400304</v>
+        <v>-0.6102251472165392</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -1779,7 +1780,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-1.198057799979097</v>
+        <v>-1.198060262302107</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1795,7 +1796,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.1474808481119823</v>
+        <v>0.1474807550235084</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1811,7 +1812,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>-0.02680421039565317</v>
+        <v>-0.02680414557239885</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -1827,7 +1828,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-0.09779437179987838</v>
+        <v>-0.09779415212066667</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -1843,7 +1844,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>-0.06005031780315306</v>
+        <v>-0.06005019859226479</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -1859,7 +1860,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>-0.02370085576838932</v>
+        <v>-0.02370079469493191</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -1875,7 +1876,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.02128540594861406</v>
+        <v>0.02128520897668196</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -1891,10 +1892,10 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4.716185427064423e-05</v>
+        <v>4.71620788751459e-05</v>
       </c>
       <c r="D65" t="n">
-        <v>5.243029858672213e-154</v>
+        <v>5.23596334384768e-154</v>
       </c>
     </row>
     <row r="66">
@@ -1907,10 +1908,10 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>-5.653477516853744e-06</v>
+        <v>-5.654476257804797e-06</v>
       </c>
       <c r="D66" t="n">
-        <v>0.03559256091393709</v>
+        <v>0.0355605429557575</v>
       </c>
     </row>
     <row r="67">
@@ -1923,7 +1924,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>-0.002329175805713568</v>
+        <v>-0.002329187405619049</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>
@@ -1939,7 +1940,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.004121507305440808</v>
+        <v>0.004121510107832904</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
@@ -1955,7 +1956,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.00246058113236769</v>
+        <v>0.002460572710933473</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -1971,10 +1972,10 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0.002775293414101654</v>
+        <v>0.002775323407323782</v>
       </c>
       <c r="D70" t="n">
-        <v>4.976011985135109e-282</v>
+        <v>4.925389404856821e-282</v>
       </c>
     </row>
     <row r="71">
@@ -1987,10 +1988,10 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.002146633223681693</v>
+        <v>0.002146637480777702</v>
       </c>
       <c r="D71" t="n">
-        <v>3.415538923054319e-149</v>
+        <v>3.417493196725461e-149</v>
       </c>
     </row>
     <row r="72">
@@ -2003,7 +2004,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.006914041267739535</v>
+        <v>0.006914318613866044</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
@@ -2019,7 +2020,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.005007976111650152</v>
+        <v>0.00500797174268444</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -2551,7 +2552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2565,55 +2566,175 @@
           <t>r2</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>mape_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>val_r2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>n_rows</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>n_features</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>neworleans</t>
+          <t>losangeles</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7880986814770712</v>
+        <v>0.9999999713728623</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.006433772500249128</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.003192452145486544</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.002528394794196245</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.9999999703979306</v>
+      </c>
+      <c r="G2" t="n">
+        <v>38062</v>
+      </c>
+      <c r="H2" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>chicago</t>
+          <t>neworleans</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.6835510594477411</v>
+        <v>0.7192021624309215</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2015.302169361358</v>
+      </c>
+      <c r="D3" t="n">
+        <v>243.1707970921586</v>
+      </c>
+      <c r="E3" t="n">
+        <v>39.55922557762002</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.8275193281322268</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6558</v>
+      </c>
+      <c r="H3" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>losangeles</t>
+          <t>newyork</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4780225671563355</v>
+        <v>0.5662145365859748</v>
+      </c>
+      <c r="C4" t="n">
+        <v>120.2996531516814</v>
+      </c>
+      <c r="D4" t="n">
+        <v>65.90057583320838</v>
+      </c>
+      <c r="E4" t="n">
+        <v>31.09749921747153</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.5970007673476083</v>
+      </c>
+      <c r="G4" t="n">
+        <v>22939</v>
+      </c>
+      <c r="H4" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>austin</t>
+          <t>chicago</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4163328917460373</v>
+        <v>0.5604173027644561</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2160.087668749142</v>
+      </c>
+      <c r="D5" t="n">
+        <v>226.0410509027986</v>
+      </c>
+      <c r="E5" t="n">
+        <v>56.42470068910299</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.6766631324136975</v>
+      </c>
+      <c r="G5" t="n">
+        <v>8186</v>
+      </c>
+      <c r="H5" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>newyork</t>
+          <t>austin</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3927486038386534</v>
+        <v>0.559543485022298</v>
+      </c>
+      <c r="C6" t="n">
+        <v>128.0801934352887</v>
+      </c>
+      <c r="D6" t="n">
+        <v>65.18051822038402</v>
+      </c>
+      <c r="E6" t="n">
+        <v>30.12512348295733</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.4678969387446772</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10206</v>
+      </c>
+      <c r="H6" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="7">
@@ -2623,7 +2744,307 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2894823891058588</v>
+        <v>0.4077590931196716</v>
+      </c>
+      <c r="C7" t="n">
+        <v>93.75892577563786</v>
+      </c>
+      <c r="D7" t="n">
+        <v>53.04701831650829</v>
+      </c>
+      <c r="E7" t="n">
+        <v>25.97421675883396</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4190975506013278</v>
+      </c>
+      <c r="G7" t="n">
+        <v>8804</v>
+      </c>
+      <c r="H7" t="n">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>target_transform</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>n_rows</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n_features</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>max_depth</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>learning_rate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>n_estimators</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>subsample</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>colsample_bytree</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>val_r2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>newyork</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>log1p</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>22939</v>
+      </c>
+      <c r="D2" t="n">
+        <v>44</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G2" t="n">
+        <v>380</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.5970007673476083</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>chicago</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>log1p</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8186</v>
+      </c>
+      <c r="D3" t="n">
+        <v>44</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G3" t="n">
+        <v>380</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.6766631324136975</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>nashville</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>log1p</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>8804</v>
+      </c>
+      <c r="D4" t="n">
+        <v>44</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.4190975506013278</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>neworleans</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>log1p</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>6558</v>
+      </c>
+      <c r="D5" t="n">
+        <v>44</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G5" t="n">
+        <v>300</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.8275193281322268</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>austin</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>log1p</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10206</v>
+      </c>
+      <c r="D6" t="n">
+        <v>44</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G6" t="n">
+        <v>350</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.4678969387446772</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>losangeles</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>log1p</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>38062</v>
+      </c>
+      <c r="D7" t="n">
+        <v>42</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G7" t="n">
+        <v>300</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.9999999703979306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Push all current project updates
</commit_message>
<xml_diff>
--- a/outputs/multi_city/tables/multi_city_analysis_summary.xlsx
+++ b/outputs/multi_city/tables/multi_city_analysis_summary.xlsx
@@ -461,13 +461,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.4431450013941</v>
+        <v>3.996005040065124</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="3">
@@ -477,13 +477,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.08319622817371827</v>
+        <v>0.007111378637464942</v>
       </c>
       <c r="C3" t="n">
-        <v>4.15722547380059e-07</v>
+        <v>0.5145718117958469</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="4">
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5648283513414091</v>
+        <v>0.3558342784323932</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="5">
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.129006167927103</v>
+        <v>0.1620895077306773</v>
       </c>
       <c r="C5" t="n">
-        <v>1.768335830545145e-13</v>
+        <v>1.223619450013219e-44</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="6">
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.001758261473381694</v>
+        <v>0.03335704234457746</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9215282956727615</v>
+        <v>0.004874701988363427</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="7">
@@ -541,13 +541,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3416981393907812</v>
+        <v>0.07387898105853222</v>
       </c>
       <c r="C7" t="n">
-        <v>9.658517252542154e-175</v>
+        <v>4.870321019472392e-20</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="8">
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.5650125737472401</v>
+        <v>0.1237155309319871</v>
       </c>
       <c r="C8" t="n">
-        <v>4.845193483037293e-109</v>
+        <v>1.859320768002485e-11</v>
       </c>
       <c r="D8" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="9">
@@ -573,13 +573,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.6337375435952312</v>
+        <v>-0.4505783488792872</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="10">
@@ -589,13 +589,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.230247678578918</v>
+        <v>-0.9261662742122871</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="11">
@@ -605,13 +605,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1165488572791514</v>
+        <v>0.1269686756608868</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="12">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.01698325177185978</v>
+        <v>-0.002908624253472269</v>
       </c>
       <c r="C12" t="n">
-        <v>1.129427103253205e-19</v>
+        <v>0.02157271585645392</v>
       </c>
       <c r="D12" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="13">
@@ -637,13 +637,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.1075412741755148</v>
+        <v>-0.05494716427732355</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="14">
@@ -653,13 +653,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.05470865909877329</v>
+        <v>-0.03954222919972572</v>
       </c>
       <c r="C14" t="n">
-        <v>6.371491062526016e-248</v>
+        <v>1.933525567702424e-291</v>
       </c>
       <c r="D14" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="15">
@@ -669,13 +669,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.000105065926965753</v>
+        <v>-0.001310792216208623</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9557334698772162</v>
+        <v>0.3059878727058149</v>
       </c>
       <c r="D15" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="16">
@@ -685,13 +685,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.0226615812362542</v>
+        <v>0.04019072237995063</v>
       </c>
       <c r="C16" t="n">
-        <v>4.159980864110577e-41</v>
+        <v>1.865358995601586e-265</v>
       </c>
       <c r="D16" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="17">
@@ -701,13 +701,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0001103763536451714</v>
+        <v>-6.59324833639946e-05</v>
       </c>
       <c r="C17" t="n">
-        <v>9.245257064760728e-35</v>
+        <v>1.196679997720957e-28</v>
       </c>
       <c r="D17" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="18">
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.0001491096054682352</v>
+        <v>-1.032339003305471e-05</v>
       </c>
       <c r="C18" t="n">
-        <v>9.914300614222562e-30</v>
+        <v>0.2342638561234942</v>
       </c>
       <c r="D18" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="19">
@@ -733,13 +733,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-0.0008809916242881155</v>
+        <v>0.001081489659263734</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0001804860116022679</v>
+        <v>4.580592729035317e-12</v>
       </c>
       <c r="D19" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="20">
@@ -749,13 +749,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.004128218035713475</v>
+        <v>0.002633294857248848</v>
       </c>
       <c r="C20" t="n">
-        <v>3.990504244658425e-28</v>
+        <v>5.643481860502171e-26</v>
       </c>
       <c r="D20" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="21">
@@ -765,13 +765,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.001441859262831513</v>
+        <v>-8.800602191006435e-05</v>
       </c>
       <c r="C21" t="n">
-        <v>2.289624265130298e-08</v>
+        <v>0.6070674850416644</v>
       </c>
       <c r="D21" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="22">
@@ -781,13 +781,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.003421966833921263</v>
+        <v>0.001732765945126626</v>
       </c>
       <c r="C22" t="n">
-        <v>1.066286278457212e-20</v>
+        <v>8.675279684926216e-13</v>
       </c>
       <c r="D22" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="23">
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.0006545664605265909</v>
+        <v>0.0002764326863114899</v>
       </c>
       <c r="C23" t="n">
-        <v>0.09184630478981877</v>
+        <v>0.283508228090016</v>
       </c>
       <c r="D23" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="24">
@@ -813,13 +813,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.006478097955520199</v>
+        <v>0.0009771165951340886</v>
       </c>
       <c r="C24" t="n">
-        <v>3.161960578087814e-123</v>
+        <v>8.354087568982688e-08</v>
       </c>
       <c r="D24" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
     <row r="25">
@@ -829,13 +829,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.0004092279085984558</v>
+        <v>0.007803676086346226</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>0.5724930833741959</v>
+        <v>0.7796334573873606</v>
       </c>
     </row>
   </sheetData>
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.098536168520923</v>
+        <v>3.825160894405599</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -900,10 +900,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1256563783468891</v>
+        <v>0.09619370085329138</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>4.242274052013942e-76</v>
       </c>
     </row>
     <row r="4">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.008107732516123</v>
+        <v>0.6947973181158886</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.2907716982534794</v>
+        <v>0.3043965685656076</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -948,10 +948,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.1027353571647609</v>
+        <v>-0.006677394092548639</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.2172003704696109</v>
       </c>
     </row>
     <row r="7">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9643289834741609</v>
+        <v>0.522065379399919</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -980,10 +980,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.3287980634171106</v>
+        <v>0.2114094580997516</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>3.747700515284289e-125</v>
       </c>
     </row>
     <row r="9">
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.7432151548240213</v>
+        <v>-0.5654789110967613</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-1.456602102031923</v>
+        <v>-1.145673401621707</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.09617351918172679</v>
+        <v>0.1126756034761911</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -1044,10 +1044,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.01523129547254598</v>
+        <v>-0.009059659955227062</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1.3800684160621e-43</v>
       </c>
     </row>
     <row r="13">
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.09347326382680876</v>
+        <v>-0.05828069875042274</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.04664975299367491</v>
+        <v>-0.04572988810321021</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -1092,10 +1092,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.01201715253792646</v>
+        <v>0.005557210662544776</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>5.412551918995852e-17</v>
       </c>
     </row>
     <row r="16">
@@ -1108,10 +1108,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.08001498507698335</v>
+        <v>0.003931642887209819</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>5.975991320460639e-10</v>
       </c>
     </row>
     <row r="17">
@@ -1124,10 +1124,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-1.298390070572641e-05</v>
+        <v>-0.0001133562351220974</v>
       </c>
       <c r="D17" t="n">
-        <v>7.461393506722341e-116</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1140,10 +1140,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-3.242625837784896e-06</v>
+        <v>-1.195923239638574e-05</v>
       </c>
       <c r="D18" t="n">
-        <v>6.255039897511553e-05</v>
+        <v>0.003661727118922938</v>
       </c>
     </row>
     <row r="19">
@@ -1156,10 +1156,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.001498306710949748</v>
+        <v>0.002302954193424966</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>3.988212626000425e-225</v>
       </c>
     </row>
     <row r="20">
@@ -1172,10 +1172,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.003909228479242799</v>
+        <v>0.003163051437297781</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1.092771829251996e-160</v>
       </c>
     </row>
     <row r="21">
@@ -1188,10 +1188,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-0.001463159731015296</v>
+        <v>-0.001784335978726403</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>2.904674791940179e-111</v>
       </c>
     </row>
     <row r="22">
@@ -1204,10 +1204,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.001735742177590538</v>
+        <v>0.001207210169653194</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1.867225111400034e-27</v>
       </c>
     </row>
     <row r="23">
@@ -1220,10 +1220,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.001589155311721768</v>
+        <v>0.0006460408717430255</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>2.036885619307552e-08</v>
       </c>
     </row>
     <row r="24">
@@ -1236,10 +1236,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-0.002235278449962408</v>
+        <v>-0.002303016802571278</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>2.802518301091103e-161</v>
       </c>
     </row>
     <row r="25">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.0002993101911952945</v>
+        <v>0.006045911792107006</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4.322580066858791</v>
+        <v>3.942577244971744</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.2739778301329352</v>
+        <v>0.1606323177429658</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.7546389411436394</v>
+        <v>0.4767683548443529</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.5347723593586124</v>
+        <v>0.3477188940833003</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.1702506688889116</v>
+        <v>0.1801637391790791</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.7028449205681682</v>
+        <v>0.2257653358037714</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -1364,10 +1364,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.3250163411685207</v>
+        <v>0.1328541085746338</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>2.978565789593059e-94</v>
       </c>
     </row>
     <row r="33">
@@ -1380,7 +1380,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-0.7296513763196657</v>
+        <v>-0.4841313285985507</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1396,7 +1396,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-1.441071017748477</v>
+        <v>-1.118267793710402</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.1194714244334136</v>
+        <v>0.1350324345432767</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
@@ -1428,10 +1428,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>-0.03863548591544941</v>
+        <v>-0.01442250080978624</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>1.588525123971776e-231</v>
       </c>
     </row>
     <row r="37">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>-0.1129628195243413</v>
+        <v>-0.05809343062838934</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-0.08577292105366041</v>
+        <v>-0.06019458550132128</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -1476,10 +1476,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>-0.01484154954027872</v>
+        <v>-0.01322391487782681</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>9.747387499406942e-191</v>
       </c>
     </row>
     <row r="40">
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-0.08991745662632411</v>
+        <v>0.03248011295529807</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1508,10 +1508,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1.197972006317105e-09</v>
+        <v>-1.650195448898994e-07</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9968719706223539</v>
+        <v>0.9366779598581274</v>
       </c>
     </row>
     <row r="42">
@@ -1524,10 +1524,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>-1.632202924900517e-09</v>
+        <v>-1.015350980515528e-07</v>
       </c>
       <c r="D42" t="n">
-        <v>0.9970951521523332</v>
+        <v>0.973329435229531</v>
       </c>
     </row>
     <row r="43">
@@ -1540,10 +1540,10 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.0003828483331744792</v>
+        <v>0.001100595215788758</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>6.783193828921321e-90</v>
       </c>
     </row>
     <row r="44">
@@ -1556,10 +1556,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.002890295843826607</v>
+        <v>0.001589324218954857</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>8.707830282897158e-74</v>
       </c>
     </row>
     <row r="45">
@@ -1572,10 +1572,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>-0.0003828296958090505</v>
+        <v>-0.001099157516961213</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>3.806289759908286e-75</v>
       </c>
     </row>
     <row r="46">
@@ -1588,10 +1588,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.0005286181876726914</v>
+        <v>0.0009975077393704623</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>6.215333695145054e-32</v>
       </c>
     </row>
     <row r="47">
@@ -1604,10 +1604,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>-0.0003828396256722044</v>
+        <v>-0.0006276362591677298</v>
       </c>
       <c r="D47" t="n">
-        <v>1.299449107418606e-183</v>
+        <v>3.447927117177139e-12</v>
       </c>
     </row>
     <row r="48">
@@ -1620,10 +1620,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2.462646989442874e-05</v>
+        <v>-0.0007011198177622191</v>
       </c>
       <c r="D48" t="n">
-        <v>0.008334949213520281</v>
+        <v>4.385733556973339e-28</v>
       </c>
     </row>
     <row r="49">
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.0005360268363976128</v>
+        <v>0.007322903436726591</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4.450210973002811</v>
+        <v>4.022005863389495</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -1668,10 +1668,10 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.04564257378501679</v>
+        <v>-0.000833933925605379</v>
       </c>
       <c r="D51" t="n">
-        <v>6.076867482915123e-42</v>
+        <v>0.8041888301257945</v>
       </c>
     </row>
     <row r="52">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.2409266965108543</v>
+        <v>0.273231817602209</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
@@ -1700,10 +1700,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.09337842806030494</v>
+        <v>0.181430281269968</v>
       </c>
       <c r="D53" t="n">
-        <v>6.05304789495267e-143</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1716,10 +1716,10 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.0198663971282258</v>
+        <v>0.1151272607439751</v>
       </c>
       <c r="D54" t="n">
-        <v>1.233585939922516e-07</v>
+        <v>1.856829186064014e-206</v>
       </c>
     </row>
     <row r="55">
@@ -1732,10 +1732,10 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>-0.04914266220015406</v>
+        <v>-0.02492102538599283</v>
       </c>
       <c r="D55" t="n">
-        <v>8.564329905782184e-89</v>
+        <v>3.850343330460485e-24</v>
       </c>
     </row>
     <row r="56">
@@ -1748,10 +1748,10 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.07334089528704624</v>
+        <v>0.0004009024892184243</v>
       </c>
       <c r="D56" t="n">
-        <v>2.342623424630981e-38</v>
+        <v>0.9431066242503231</v>
       </c>
     </row>
     <row r="57">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>-0.6102251472165392</v>
+        <v>-0.4386067718478444</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-1.198060262302107</v>
+        <v>-0.9331927250726721</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.1474807550235084</v>
+        <v>0.1603189046415849</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -1812,10 +1812,10 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>-0.02680414557239885</v>
+        <v>-0.008749674312895195</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>1.330956111160866e-171</v>
       </c>
     </row>
     <row r="61">
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-0.09779415212066667</v>
+        <v>-0.06692261763839724</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>-0.06005019859226479</v>
+        <v>-0.054114778058306</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -1860,7 +1860,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>-0.02370079469493191</v>
+        <v>-0.01634020006747505</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -1876,7 +1876,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.02128520897668196</v>
+        <v>0.05366431850472964</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -1892,10 +1892,10 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4.71620788751459e-05</v>
+        <v>8.409893580141325e-09</v>
       </c>
       <c r="D65" t="n">
-        <v>5.23596334384768e-154</v>
+        <v>0.9962879595600957</v>
       </c>
     </row>
     <row r="66">
@@ -1908,10 +1908,10 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>-5.654476257804797e-06</v>
+        <v>2.858700359764654e-09</v>
       </c>
       <c r="D66" t="n">
-        <v>0.0355605429557575</v>
+        <v>0.9991211092609698</v>
       </c>
     </row>
     <row r="67">
@@ -1924,10 +1924,10 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>-0.002329187405619049</v>
+        <v>-0.0003799116228151433</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>1.807459335204535e-13</v>
       </c>
     </row>
     <row r="68">
@@ -1940,10 +1940,10 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.004121510107832904</v>
+        <v>0.002395511294238872</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>9.517233350502641e-192</v>
       </c>
     </row>
     <row r="69">
@@ -1956,10 +1956,10 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.002460572710933473</v>
+        <v>0.0003803121207113236</v>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>9.538873571331845e-12</v>
       </c>
     </row>
     <row r="70">
@@ -1972,10 +1972,10 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0.002775323407323782</v>
+        <v>0.001722658060032245</v>
       </c>
       <c r="D70" t="n">
-        <v>4.925389404856821e-282</v>
+        <v>3.804233606170534e-108</v>
       </c>
     </row>
     <row r="71">
@@ -1988,10 +1988,10 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.002146637480777702</v>
+        <v>0.0003799089765834651</v>
       </c>
       <c r="D71" t="n">
-        <v>3.417493196725461e-149</v>
+        <v>7.575204932284816e-06</v>
       </c>
     </row>
     <row r="72">
@@ -2004,10 +2004,10 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.006914318613866044</v>
+        <v>0.000381782016603438</v>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
+        <v>1.252971765245167e-10</v>
       </c>
     </row>
     <row r="73">
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.00500797174268444</v>
+        <v>0.009888564968530744</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
@@ -2094,13 +2094,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>929.4854183669647</v>
+        <v>970.0099337593601</v>
       </c>
       <c r="E2" t="n">
-        <v>1.10506937914719e-198</v>
+        <v>1.867861795531417e-207</v>
       </c>
       <c r="F2" t="n">
-        <v>1.10506937914719e-198</v>
+        <v>1.867861795531417e-207</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
@@ -2123,13 +2123,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>42047341</v>
+        <v>41247765</v>
       </c>
       <c r="E3" t="n">
-        <v>1.238137724395615e-14</v>
+        <v>4.556167045516401e-13</v>
       </c>
       <c r="F3" t="n">
-        <v>2.321508233241778e-14</v>
+        <v>6.21295506206782e-13</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -2152,13 +2152,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>226704452</v>
+        <v>222447850</v>
       </c>
       <c r="E4" t="n">
-        <v>5.469108875184265e-13</v>
+        <v>5.367966864275134e-19</v>
       </c>
       <c r="F4" t="n">
-        <v>9.115181458640441e-13</v>
+        <v>1.006493787051588e-18</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -2181,13 +2181,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>41881902</v>
+        <v>41003299.5</v>
       </c>
       <c r="E5" t="n">
-        <v>1.329339139500949e-65</v>
+        <v>4.57650660844445e-76</v>
       </c>
       <c r="F5" t="n">
-        <v>4.985021773128558e-65</v>
+        <v>2.288253304222226e-75</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -2210,16 +2210,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>37774185.5</v>
+        <v>37088493</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01087622169252149</v>
+        <v>0.09834960919189586</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01087622169252149</v>
+        <v>0.09834960919189586</v>
       </c>
       <c r="G6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2239,13 +2239,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>192065574.5</v>
+        <v>188708159.5</v>
       </c>
       <c r="E7" t="n">
-        <v>7.808894132680704e-06</v>
+        <v>0.0003281864567505067</v>
       </c>
       <c r="F7" t="n">
-        <v>9.010262460785427e-06</v>
+        <v>0.0003516283465184001</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -2268,13 +2268,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>208656364.5</v>
+        <v>203222404.5</v>
       </c>
       <c r="E8" t="n">
-        <v>4.86987204564723e-32</v>
+        <v>2.547504208669743e-21</v>
       </c>
       <c r="F8" t="n">
-        <v>1.043544009781549e-31</v>
+        <v>5.458937590006592e-21</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -2297,13 +2297,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>38128856.5</v>
+        <v>37007265</v>
       </c>
       <c r="E9" t="n">
-        <v>3.499958699648332e-10</v>
+        <v>5.322855849895665e-16</v>
       </c>
       <c r="F9" t="n">
-        <v>4.772670954065907e-10</v>
+        <v>8.871426416492774e-16</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -2326,13 +2326,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>33622197.5</v>
+        <v>32740079</v>
       </c>
       <c r="E10" t="n">
-        <v>1.179187941596919e-08</v>
+        <v>6.341188338100575e-10</v>
       </c>
       <c r="F10" t="n">
-        <v>1.473984926996149e-08</v>
+        <v>7.92648542262572e-10</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -2355,13 +2355,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>169666727</v>
+        <v>165370242.5</v>
       </c>
       <c r="E11" t="n">
-        <v>1.620515906351819e-46</v>
+        <v>4.354484366137154e-38</v>
       </c>
       <c r="F11" t="n">
-        <v>4.051289765879548e-46</v>
+        <v>1.088621091534288e-37</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
@@ -2387,10 +2387,10 @@
         <v>184530396</v>
       </c>
       <c r="E12" t="n">
-        <v>7.83111576996665e-120</v>
+        <v>8.190884493328381e-122</v>
       </c>
       <c r="F12" t="n">
-        <v>5.873336827474987e-119</v>
+        <v>6.143163369996285e-121</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
@@ -2416,10 +2416,10 @@
         <v>172259848</v>
       </c>
       <c r="E13" t="n">
-        <v>1.254355105407153e-05</v>
+        <v>4.467898182675336e-13</v>
       </c>
       <c r="F13" t="n">
-        <v>1.343951898650521e-05</v>
+        <v>6.21295506206782e-13</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
@@ -2445,10 +2445,10 @@
         <v>863714891</v>
       </c>
       <c r="E14" t="n">
-        <v>2.252951708146588e-66</v>
+        <v>3.253949087500072e-73</v>
       </c>
       <c r="F14" t="n">
-        <v>1.126475854073294e-65</v>
+        <v>1.220230907812527e-72</v>
       </c>
       <c r="G14" t="b">
         <v>1</v>
@@ -2471,13 +2471,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>39136734.5</v>
+        <v>39216861.5</v>
       </c>
       <c r="E15" t="n">
-        <v>7.750415610549594e-48</v>
+        <v>5.424897452683327e-63</v>
       </c>
       <c r="F15" t="n">
-        <v>2.325124683164878e-47</v>
+        <v>1.627469235804998e-62</v>
       </c>
       <c r="G15" t="b">
         <v>1</v>
@@ -2500,13 +2500,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>196160897</v>
+        <v>196553450</v>
       </c>
       <c r="E16" t="n">
-        <v>3.025099717967735e-147</v>
+        <v>2.267240492267547e-155</v>
       </c>
       <c r="F16" t="n">
-        <v>4.537649576951603e-146</v>
+        <v>3.40086073840132e-154</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
@@ -2529,13 +2529,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>139202809.5</v>
+        <v>134692288</v>
       </c>
       <c r="E17" t="n">
-        <v>2.415432578872589e-11</v>
+        <v>1.246452731060919e-06</v>
       </c>
       <c r="F17" t="n">
-        <v>3.623148868308884e-11</v>
+        <v>1.438214689685676e-06</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
@@ -2552,7 +2552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2600,169 +2600,141 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>losangeles</t>
+          <t>newyork</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9999999713728623</v>
+        <v>0.6919305901500099</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006433772500249128</v>
+        <v>101.2943236276103</v>
       </c>
       <c r="D2" t="n">
-        <v>0.003192452145486544</v>
+        <v>55.53600257144254</v>
       </c>
       <c r="E2" t="n">
-        <v>0.002528394794196245</v>
+        <v>26.6833096733373</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9999999703979306</v>
+        <v>0.6907548926537888</v>
       </c>
       <c r="G2" t="n">
-        <v>38062</v>
+        <v>20398</v>
       </c>
       <c r="H2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>neworleans</t>
+          <t>chicago</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7192021624309215</v>
+        <v>0.6286093194609854</v>
       </c>
       <c r="C3" t="n">
-        <v>2015.302169361358</v>
+        <v>89.41862603633744</v>
       </c>
       <c r="D3" t="n">
-        <v>243.1707970921586</v>
+        <v>50.71118238566336</v>
       </c>
       <c r="E3" t="n">
-        <v>39.55922557762002</v>
+        <v>26.86794711884902</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8275193281322268</v>
+        <v>0.583222015506198</v>
       </c>
       <c r="G3" t="n">
-        <v>6558</v>
+        <v>7562</v>
       </c>
       <c r="H3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>newyork</t>
+          <t>nashville</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5662145365859748</v>
+        <v>0.5781518342190767</v>
       </c>
       <c r="C4" t="n">
-        <v>120.2996531516814</v>
+        <v>95.62002957177064</v>
       </c>
       <c r="D4" t="n">
-        <v>65.90057583320838</v>
+        <v>54.50512185412673</v>
       </c>
       <c r="E4" t="n">
-        <v>31.09749921747153</v>
+        <v>25.86944537823018</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5970007673476083</v>
+        <v>0.5456005137691536</v>
       </c>
       <c r="G4" t="n">
-        <v>22939</v>
+        <v>6487</v>
       </c>
       <c r="H4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>chicago</t>
+          <t>austin</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5604173027644561</v>
+        <v>0.5462709860898746</v>
       </c>
       <c r="C5" t="n">
-        <v>2160.087668749142</v>
+        <v>116.0300498312769</v>
       </c>
       <c r="D5" t="n">
-        <v>226.0410509027986</v>
+        <v>62.51168174913446</v>
       </c>
       <c r="E5" t="n">
-        <v>56.42470068910299</v>
+        <v>31.0536945958821</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6766631324136975</v>
+        <v>0.5497212178451871</v>
       </c>
       <c r="G5" t="n">
-        <v>8186</v>
+        <v>10108</v>
       </c>
       <c r="H5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>austin</t>
+          <t>neworleans</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.559543485022298</v>
+        <v>0.455435371243046</v>
       </c>
       <c r="C6" t="n">
-        <v>128.0801934352887</v>
+        <v>112.2615117372473</v>
       </c>
       <c r="D6" t="n">
-        <v>65.18051822038402</v>
+        <v>61.48446370198298</v>
       </c>
       <c r="E6" t="n">
-        <v>30.12512348295733</v>
+        <v>32.86087368520797</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4678969387446772</v>
+        <v>0.5023806888656366</v>
       </c>
       <c r="G6" t="n">
-        <v>10206</v>
+        <v>6035</v>
       </c>
       <c r="H6" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>nashville</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.4077590931196716</v>
-      </c>
-      <c r="C7" t="n">
-        <v>93.75892577563786</v>
-      </c>
-      <c r="D7" t="n">
-        <v>53.04701831650829</v>
-      </c>
-      <c r="E7" t="n">
-        <v>25.97421675883396</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.4190975506013278</v>
-      </c>
-      <c r="G7" t="n">
-        <v>8804</v>
-      </c>
-      <c r="H7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2776,7 +2748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2843,10 +2815,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22939</v>
+        <v>20398</v>
       </c>
       <c r="D2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
@@ -2864,7 +2836,7 @@
         <v>0.95</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5970007673476083</v>
+        <v>0.6907548926537888</v>
       </c>
     </row>
     <row r="3">
@@ -2879,28 +2851,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8186</v>
+        <v>7562</v>
       </c>
       <c r="D3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>0.04</v>
       </c>
       <c r="G3" t="n">
-        <v>380</v>
+        <v>450</v>
       </c>
       <c r="H3" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="I3" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6766631324136975</v>
+        <v>0.583222015506198</v>
       </c>
     </row>
     <row r="4">
@@ -2915,19 +2887,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8804</v>
+        <v>6487</v>
       </c>
       <c r="D4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="G4" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="H4" t="n">
         <v>0.9</v>
@@ -2936,7 +2908,7 @@
         <v>0.9</v>
       </c>
       <c r="J4" t="n">
-        <v>0.4190975506013278</v>
+        <v>0.5456005137691536</v>
       </c>
     </row>
     <row r="5">
@@ -2951,28 +2923,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6558</v>
+        <v>6035</v>
       </c>
       <c r="D5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="G5" t="n">
-        <v>300</v>
+        <v>380</v>
       </c>
       <c r="H5" t="n">
         <v>0.85</v>
       </c>
       <c r="I5" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8275193281322268</v>
+        <v>0.5023806888656366</v>
       </c>
     </row>
     <row r="6">
@@ -2987,19 +2959,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10206</v>
+        <v>10108</v>
       </c>
       <c r="D6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="G6" t="n">
-        <v>350</v>
+        <v>450</v>
       </c>
       <c r="H6" t="n">
         <v>0.9</v>
@@ -3008,43 +2980,7 @@
         <v>0.9</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4678969387446772</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>losangeles</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>log1p</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>38062</v>
-      </c>
-      <c r="D7" t="n">
-        <v>42</v>
-      </c>
-      <c r="E7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G7" t="n">
-        <v>300</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.9999999703979306</v>
+        <v>0.5497212178451871</v>
       </c>
     </row>
   </sheetData>

</xml_diff>